<commit_message>
Atualiza BACKLOG.xlsx - Issues da Onda 2 preenchidas
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{BDDC8BC0-41D6-4ABA-8A9E-CEE4CCC72C13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E72C77FE-03F3-4ECB-BA7A-7160974D1D05}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="13_ncr:1_{BDDC8BC0-41D6-4ABA-8A9E-CEE4CCC72C13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BFB2501E-25BE-4DC0-8F4B-3198353F61FD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -207,109 +207,109 @@
     <t>Definir estrutura da interface para criação e edição dos critérios de avaliação de uma vaga</t>
   </si>
   <si>
+    <t>#35</t>
+  </si>
+  <si>
+    <t>T10</t>
+  </si>
+  <si>
+    <t>Implementar interface para cadastrar, editar e excluir critérios de avaliação da vaga</t>
+  </si>
+  <si>
+    <t>#36</t>
+  </si>
+  <si>
+    <t>T11</t>
+  </si>
+  <si>
+    <t>Relacionar o perfil estruturado do candidato aos critérios de avaliação da vaga</t>
+  </si>
+  <si>
+    <t>#28</t>
+  </si>
+  <si>
+    <t>T12</t>
+  </si>
+  <si>
+    <t>Criar persistência e APIs para critérios de avaliação vinculados à vaga</t>
+  </si>
+  <si>
+    <t>#29</t>
+  </si>
+  <si>
+    <t>T13</t>
+  </si>
+  <si>
+    <t>F11</t>
+  </si>
+  <si>
+    <t>Definir interface e fluxo para registro e consulta da entrevista do candidato</t>
+  </si>
+  <si>
+    <t>#32</t>
+  </si>
+  <si>
+    <t>T14</t>
+  </si>
+  <si>
+    <t>Implementar registro e consulta dos dados da entrevista</t>
+  </si>
+  <si>
+    <t>#33</t>
+  </si>
+  <si>
+    <t>T15</t>
+  </si>
+  <si>
+    <t>Criar persistência e APIs para registro e recuperação das entrevistas</t>
+  </si>
+  <si>
+    <t>#26</t>
+  </si>
+  <si>
+    <t>T16</t>
+  </si>
+  <si>
+    <t>F12</t>
+  </si>
+  <si>
+    <t>Implementar atualização do perfil do candidato com informações provenientes da entrevista</t>
+  </si>
+  <si>
+    <t>#30</t>
+  </si>
+  <si>
+    <t>T17</t>
+  </si>
+  <si>
+    <t>Implementar edição e visualização do perfil enriquecido após a entrevista</t>
+  </si>
+  <si>
+    <t>#37</t>
+  </si>
+  <si>
+    <t>T18</t>
+  </si>
+  <si>
+    <t>Definir regras de consolidação entre informações do currículo e informações da entrevista</t>
+  </si>
+  <si>
+    <t>#38</t>
+  </si>
+  <si>
+    <t>T19</t>
+  </si>
+  <si>
+    <t>Onda 3</t>
+  </si>
+  <si>
+    <t>F09</t>
+  </si>
+  <si>
+    <t>Criar spike técnico para avaliar integração com as plataformas externas previstas</t>
+  </si>
+  <si>
     <t>--</t>
-  </si>
-  <si>
-    <t>#35</t>
-  </si>
-  <si>
-    <t>T10</t>
-  </si>
-  <si>
-    <t>Implementar interface para cadastrar, editar e excluir critérios de avaliação da vaga</t>
-  </si>
-  <si>
-    <t>#36</t>
-  </si>
-  <si>
-    <t>T11</t>
-  </si>
-  <si>
-    <t>Relacionar o perfil estruturado do candidato aos critérios de avaliação da vaga</t>
-  </si>
-  <si>
-    <t>#28</t>
-  </si>
-  <si>
-    <t>T12</t>
-  </si>
-  <si>
-    <t>Criar persistência e APIs para critérios de avaliação vinculados à vaga</t>
-  </si>
-  <si>
-    <t>#29</t>
-  </si>
-  <si>
-    <t>T13</t>
-  </si>
-  <si>
-    <t>F11</t>
-  </si>
-  <si>
-    <t>Definir interface e fluxo para registro e consulta da entrevista do candidato</t>
-  </si>
-  <si>
-    <t>#32</t>
-  </si>
-  <si>
-    <t>T14</t>
-  </si>
-  <si>
-    <t>Implementar registro e consulta dos dados da entrevista</t>
-  </si>
-  <si>
-    <t>#33</t>
-  </si>
-  <si>
-    <t>T15</t>
-  </si>
-  <si>
-    <t>Criar persistência e APIs para registro e recuperação das entrevistas</t>
-  </si>
-  <si>
-    <t>#26</t>
-  </si>
-  <si>
-    <t>T16</t>
-  </si>
-  <si>
-    <t>F12</t>
-  </si>
-  <si>
-    <t>Implementar atualização do perfil do candidato com informações provenientes da entrevista</t>
-  </si>
-  <si>
-    <t>#30</t>
-  </si>
-  <si>
-    <t>T17</t>
-  </si>
-  <si>
-    <t>Implementar edição e visualização do perfil enriquecido após a entrevista</t>
-  </si>
-  <si>
-    <t>#37</t>
-  </si>
-  <si>
-    <t>T18</t>
-  </si>
-  <si>
-    <t>Definir regras de consolidação entre informações do currículo e informações da entrevista</t>
-  </si>
-  <si>
-    <t>#38</t>
-  </si>
-  <si>
-    <t>T19</t>
-  </si>
-  <si>
-    <t>Onda 3</t>
-  </si>
-  <si>
-    <t>F09</t>
-  </si>
-  <si>
-    <t>Criar spike técnico para avaliar integração com as plataformas externas previstas</t>
   </si>
   <si>
     <t>T20</t>
@@ -1141,7 +1141,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:H136"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1222,7 +1221,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" hidden="1">
+    <row r="5" spans="1:8" ht="30">
       <c r="A5" s="14" t="s">
         <v>14</v>
       </c>
@@ -1248,7 +1247,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="30" hidden="1">
+    <row r="6" spans="1:8" ht="30">
       <c r="A6" s="14" t="s">
         <v>22</v>
       </c>
@@ -1274,7 +1273,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="30" hidden="1">
+    <row r="7" spans="1:8" ht="30">
       <c r="A7" s="14" t="s">
         <v>27</v>
       </c>
@@ -1300,7 +1299,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="30" hidden="1">
+    <row r="8" spans="1:8" ht="30">
       <c r="A8" s="14" t="s">
         <v>32</v>
       </c>
@@ -1326,7 +1325,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30" hidden="1">
+    <row r="9" spans="1:8" ht="30">
       <c r="A9" s="14" t="s">
         <v>36</v>
       </c>
@@ -1352,7 +1351,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:8" hidden="1">
+    <row r="10" spans="1:8">
       <c r="A10" s="14" t="s">
         <v>41</v>
       </c>
@@ -1378,7 +1377,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:8" hidden="1">
+    <row r="11" spans="1:8">
       <c r="A11" s="14" t="s">
         <v>44</v>
       </c>
@@ -1404,7 +1403,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:8" hidden="1">
+    <row r="12" spans="1:8">
       <c r="A12" s="14" t="s">
         <v>47</v>
       </c>
@@ -1450,15 +1449,15 @@
         <v>19</v>
       </c>
       <c r="G13" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="H13" s="11" t="s">
         <v>55</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B14" s="15" t="s">
         <v>52</v>
@@ -1470,21 +1469,21 @@
         <v>23</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F14" s="14" t="s">
         <v>25</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="H14" s="11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>52</v>
@@ -1496,7 +1495,7 @@
         <v>28</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F15" s="14" t="s">
         <v>25</v>
@@ -1505,12 +1504,12 @@
         <v>30</v>
       </c>
       <c r="H15" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="18" customHeight="1">
       <c r="A16" s="14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B16" s="15" t="s">
         <v>52</v>
@@ -1522,7 +1521,7 @@
         <v>28</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F16" s="14" t="s">
         <v>25</v>
@@ -1531,24 +1530,24 @@
         <v>30</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1">
       <c r="A17" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B17" s="15" t="s">
         <v>52</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D17" s="14" t="s">
         <v>17</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F17" s="14" t="s">
         <v>19</v>
@@ -1557,24 +1556,24 @@
         <v>20</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B18" s="15" t="s">
         <v>52</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D18" s="14" t="s">
         <v>23</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F18" s="14" t="s">
         <v>25</v>
@@ -1583,24 +1582,24 @@
         <v>20</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B19" s="15" t="s">
         <v>52</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D19" s="14" t="s">
         <v>28</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F19" s="14" t="s">
         <v>25</v>
@@ -1609,24 +1608,24 @@
         <v>30</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="30.75">
       <c r="A20" s="14" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B20" s="15" t="s">
         <v>52</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D20" s="14" t="s">
         <v>28</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F20" s="14" t="s">
         <v>25</v>
@@ -1635,96 +1634,96 @@
         <v>30</v>
       </c>
       <c r="H20" s="11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="15.95" customHeight="1">
       <c r="A21" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B21" s="15" t="s">
         <v>52</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D21" s="14" t="s">
         <v>23</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F21" s="14" t="s">
         <v>25</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="30.75">
       <c r="A22" s="14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>52</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D22" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E22" s="14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F22" s="14" t="s">
         <v>19</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="H22" s="13" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" s="14" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" hidden="1">
-      <c r="A23" s="14" t="s">
+      <c r="B23" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="B23" s="15" t="s">
+      <c r="C23" s="14" t="s">
         <v>87</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>88</v>
       </c>
       <c r="D23" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F23" s="14" t="s">
         <v>25</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="30" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="30">
       <c r="A24" s="14" t="s">
         <v>90</v>
       </c>
       <c r="B24" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="C24" s="14" t="s">
         <v>87</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>88</v>
       </c>
       <c r="D24" s="14" t="s">
         <v>28</v>
@@ -1736,21 +1735,21 @@
         <v>25</v>
       </c>
       <c r="G24" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="30" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="30">
       <c r="A25" s="14" t="s">
         <v>92</v>
       </c>
       <c r="B25" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="C25" s="14" t="s">
         <v>87</v>
-      </c>
-      <c r="C25" s="14" t="s">
-        <v>88</v>
       </c>
       <c r="D25" s="14" t="s">
         <v>23</v>
@@ -1762,18 +1761,18 @@
         <v>19</v>
       </c>
       <c r="G25" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="15.95" hidden="1" customHeight="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="15.95" customHeight="1">
       <c r="A26" s="14" t="s">
         <v>94</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C26" s="14" t="s">
         <v>95</v>
@@ -1788,18 +1787,18 @@
         <v>19</v>
       </c>
       <c r="G26" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H26" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="30" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="30">
       <c r="A27" s="14" t="s">
         <v>97</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C27" s="14" t="s">
         <v>95</v>
@@ -1820,12 +1819,12 @@
         <v>99</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="30" hidden="1">
+    <row r="28" spans="1:8" ht="30">
       <c r="A28" s="14" t="s">
         <v>100</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C28" s="14" t="s">
         <v>95</v>
@@ -1840,18 +1839,18 @@
         <v>25</v>
       </c>
       <c r="G28" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="30" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="30">
       <c r="A29" s="14" t="s">
         <v>102</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C29" s="14" t="s">
         <v>103</v>
@@ -1866,18 +1865,18 @@
         <v>19</v>
       </c>
       <c r="G29" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="27" hidden="1" customHeight="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="27" customHeight="1">
       <c r="A30" s="14" t="s">
         <v>105</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C30" s="14" t="s">
         <v>103</v>
@@ -1892,18 +1891,18 @@
         <v>25</v>
       </c>
       <c r="G30" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="27.75" hidden="1" customHeight="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="27.75" customHeight="1">
       <c r="A31" s="14" t="s">
         <v>107</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C31" s="14" t="s">
         <v>103</v>
@@ -1924,7 +1923,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="32" spans="1:8" hidden="1">
+    <row r="32" spans="1:8">
       <c r="A32" s="14" t="s">
         <v>109</v>
       </c>
@@ -1944,13 +1943,13 @@
         <v>25</v>
       </c>
       <c r="G32" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" ht="30" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="30">
       <c r="A33" s="14" t="s">
         <v>113</v>
       </c>
@@ -1970,13 +1969,13 @@
         <v>25</v>
       </c>
       <c r="G33" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" ht="30" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="30">
       <c r="A34" s="14" t="s">
         <v>115</v>
       </c>
@@ -1996,13 +1995,13 @@
         <v>25</v>
       </c>
       <c r="G34" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" ht="30" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="30">
       <c r="A35" s="14" t="s">
         <v>117</v>
       </c>
@@ -2022,13 +2021,13 @@
         <v>25</v>
       </c>
       <c r="G35" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" ht="30" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="30">
       <c r="A36" s="14" t="s">
         <v>119</v>
       </c>
@@ -2048,13 +2047,13 @@
         <v>19</v>
       </c>
       <c r="G36" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" ht="30" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="30">
       <c r="A37" s="14" t="s">
         <v>122</v>
       </c>
@@ -2074,13 +2073,13 @@
         <v>25</v>
       </c>
       <c r="G37" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
       <c r="A38" s="14" t="s">
         <v>124</v>
       </c>
@@ -2100,13 +2099,13 @@
         <v>25</v>
       </c>
       <c r="G38" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H38" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
       <c r="A39" s="14" t="s">
         <v>126</v>
       </c>
@@ -2126,13 +2125,13 @@
         <v>19</v>
       </c>
       <c r="G39" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
       <c r="A40" s="14" t="s">
         <v>129</v>
       </c>
@@ -2152,13 +2151,13 @@
         <v>19</v>
       </c>
       <c r="G40" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H40" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
       <c r="A41" s="14" t="s">
         <v>131</v>
       </c>
@@ -2178,13 +2177,13 @@
         <v>19</v>
       </c>
       <c r="G41" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H41" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
       <c r="A42" s="14" t="s">
         <v>133</v>
       </c>
@@ -2204,13 +2203,13 @@
         <v>19</v>
       </c>
       <c r="G42" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H42" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
       <c r="A43" s="14" t="s">
         <v>137</v>
       </c>
@@ -2230,13 +2229,13 @@
         <v>19</v>
       </c>
       <c r="G43" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H43" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
       <c r="A44" s="14" t="s">
         <v>139</v>
       </c>
@@ -2256,13 +2255,13 @@
         <v>19</v>
       </c>
       <c r="G44" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H44" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" ht="30" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="30">
       <c r="A45" s="14" t="s">
         <v>141</v>
       </c>
@@ -2282,13 +2281,13 @@
         <v>19</v>
       </c>
       <c r="G45" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H45" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" ht="30" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="30">
       <c r="A46" s="14" t="s">
         <v>144</v>
       </c>
@@ -2308,13 +2307,13 @@
         <v>25</v>
       </c>
       <c r="G46" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H46" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
       <c r="A47" s="14" t="s">
         <v>146</v>
       </c>
@@ -2334,13 +2333,13 @@
         <v>25</v>
       </c>
       <c r="G47" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H47" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
       <c r="A48" s="14" t="s">
         <v>148</v>
       </c>
@@ -2360,13 +2359,13 @@
         <v>19</v>
       </c>
       <c r="G48" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H48" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
       <c r="A49" s="14" t="s">
         <v>151</v>
       </c>
@@ -2386,13 +2385,13 @@
         <v>25</v>
       </c>
       <c r="G49" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H49" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" ht="30" hidden="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="30">
       <c r="A50" s="14" t="s">
         <v>153</v>
       </c>
@@ -2412,10 +2411,10 @@
         <v>25</v>
       </c>
       <c r="G50" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="H50" s="13" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -3280,11 +3279,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A4:H50" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="Onda 2"/>
-      </filters>
-    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:H50">
       <sortCondition ref="B4:B50"/>
     </sortState>
@@ -3749,6 +3743,14 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="d90de4e3-1570-4373-8742-4e5b70768c2c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -3757,22 +3759,14 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="d90de4e3-1570-4373-8742-4e5b70768c2c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F54BD295-47E6-4D5E-AB8C-AB6A369202DB}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0FA79B10-923E-46FD-992E-6B2FB513113C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8C9EAED-E792-4EBD-8FE5-A88413F06C36}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8C9EAED-E792-4EBD-8FE5-A88413F06C36}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0FA79B10-923E-46FD-992E-6B2FB513113C}"/>
 </file>
</xml_diff>

<commit_message>
Atualiza BACKLOG.xlsx - Issues da Onda 3 preenchidas
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30621"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="13_ncr:1_{BDDC8BC0-41D6-4ABA-8A9E-CEE4CCC72C13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BFB2501E-25BE-4DC0-8F4B-3198353F61FD}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="13_ncr:1_{BDDC8BC0-41D6-4ABA-8A9E-CEE4CCC72C13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11F78EB9-6E27-44B8-83A0-6223A007AC91}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="189">
   <si>
     <t>BACKLOG DO PRODUTO — Todas as Ondas até o MVP</t>
   </si>
@@ -309,13 +309,19 @@
     <t>Criar spike técnico para avaliar integração com as plataformas externas previstas</t>
   </si>
   <si>
+    <t>#41</t>
+  </si>
+  <si>
+    <t>T20</t>
+  </si>
+  <si>
+    <t>Implementar integração e importação de currículos a partir das plataformas externas selecionadas</t>
+  </si>
+  <si>
     <t>--</t>
   </si>
   <si>
-    <t>T20</t>
-  </si>
-  <si>
-    <t>Implementar integração e importação de currículos a partir das plataformas externas selecionadas</t>
+    <t>#42</t>
   </si>
   <si>
     <t>T21</t>
@@ -324,6 +330,9 @@
     <t>Implementar interface para iniciar a importação e acompanhar o resultado da integração</t>
   </si>
   <si>
+    <t>#43</t>
+  </si>
+  <si>
     <t>T22</t>
   </si>
   <si>
@@ -333,6 +342,9 @@
     <t>Definir apresentação dos critérios e resultados da avaliação comportamental</t>
   </si>
   <si>
+    <t>#44</t>
+  </si>
+  <si>
     <t>T23</t>
   </si>
   <si>
@@ -348,6 +360,9 @@
     <t>Implementar visualização dos resultados da avaliação comportamental por candidato</t>
   </si>
   <si>
+    <t>#45</t>
+  </si>
+  <si>
     <t>T25</t>
   </si>
   <si>
@@ -357,10 +372,16 @@
     <t>Definir interface para acompanhamento da adaptação técnica e comportamental do novo funcionário</t>
   </si>
   <si>
+    <t>#46</t>
+  </si>
+  <si>
     <t>T26</t>
   </si>
   <si>
     <t>Implementar registro e visualização do acompanhamento da adaptação do funcionário</t>
+  </si>
+  <si>
+    <t>#47</t>
   </si>
   <si>
     <t>T27</t>
@@ -1141,6 +1162,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:H136"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1221,7 +1243,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30">
+    <row r="5" spans="1:8" ht="30" hidden="1">
       <c r="A5" s="14" t="s">
         <v>14</v>
       </c>
@@ -1247,7 +1269,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="30">
+    <row r="6" spans="1:8" ht="30" hidden="1">
       <c r="A6" s="14" t="s">
         <v>22</v>
       </c>
@@ -1273,7 +1295,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="30">
+    <row r="7" spans="1:8" ht="30" hidden="1">
       <c r="A7" s="14" t="s">
         <v>27</v>
       </c>
@@ -1299,7 +1321,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="30">
+    <row r="8" spans="1:8" ht="30" hidden="1">
       <c r="A8" s="14" t="s">
         <v>32</v>
       </c>
@@ -1325,7 +1347,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30">
+    <row r="9" spans="1:8" ht="30" hidden="1">
       <c r="A9" s="14" t="s">
         <v>36</v>
       </c>
@@ -1351,7 +1373,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" hidden="1">
       <c r="A10" s="14" t="s">
         <v>41</v>
       </c>
@@ -1377,7 +1399,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" hidden="1">
       <c r="A11" s="14" t="s">
         <v>44</v>
       </c>
@@ -1403,7 +1425,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" hidden="1">
       <c r="A12" s="14" t="s">
         <v>47</v>
       </c>
@@ -1429,7 +1451,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30.75">
+    <row r="13" spans="1:8" ht="30.75" hidden="1">
       <c r="A13" s="14" t="s">
         <v>51</v>
       </c>
@@ -1455,7 +1477,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" hidden="1">
       <c r="A14" s="14" t="s">
         <v>56</v>
       </c>
@@ -1481,7 +1503,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" hidden="1">
       <c r="A15" s="14" t="s">
         <v>59</v>
       </c>
@@ -1507,7 +1529,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="18" customHeight="1">
+    <row r="16" spans="1:8" ht="18" hidden="1" customHeight="1">
       <c r="A16" s="14" t="s">
         <v>62</v>
       </c>
@@ -1533,7 +1555,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="18" customHeight="1">
+    <row r="17" spans="1:8" ht="18" hidden="1" customHeight="1">
       <c r="A17" s="14" t="s">
         <v>65</v>
       </c>
@@ -1559,7 +1581,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:8" hidden="1">
       <c r="A18" s="14" t="s">
         <v>69</v>
       </c>
@@ -1585,7 +1607,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" hidden="1">
       <c r="A19" s="14" t="s">
         <v>72</v>
       </c>
@@ -1611,7 +1633,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="30.75">
+    <row r="20" spans="1:8" ht="30.75" hidden="1">
       <c r="A20" s="14" t="s">
         <v>75</v>
       </c>
@@ -1637,7 +1659,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15.95" customHeight="1">
+    <row r="21" spans="1:8" ht="15.95" hidden="1" customHeight="1">
       <c r="A21" s="14" t="s">
         <v>79</v>
       </c>
@@ -1663,7 +1685,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30.75">
+    <row r="22" spans="1:8" ht="30.75" hidden="1">
       <c r="A22" s="14" t="s">
         <v>82</v>
       </c>
@@ -1709,13 +1731,13 @@
         <v>25</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>89</v>
+        <v>49</v>
       </c>
       <c r="H23" s="13" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="30">
+    <row r="24" spans="1:8" ht="30.75">
       <c r="A24" s="14" t="s">
         <v>90</v>
       </c>
@@ -1735,15 +1757,15 @@
         <v>25</v>
       </c>
       <c r="G24" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="30">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="30.75">
       <c r="A25" s="14" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B25" s="15" t="s">
         <v>86</v>
@@ -1755,59 +1777,59 @@
         <v>23</v>
       </c>
       <c r="E25" s="14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F25" s="14" t="s">
         <v>19</v>
       </c>
       <c r="G25" s="13" t="s">
-        <v>89</v>
+        <v>49</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="15.95" customHeight="1">
       <c r="A26" s="14" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B26" s="15" t="s">
         <v>86</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D26" s="14" t="s">
         <v>17</v>
       </c>
       <c r="E26" s="14" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="F26" s="14" t="s">
         <v>19</v>
       </c>
       <c r="G26" s="13" t="s">
-        <v>89</v>
+        <v>49</v>
       </c>
       <c r="H26" s="13" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="30">
       <c r="A27" s="14" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B27" s="15" t="s">
         <v>86</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D27" s="14" t="s">
         <v>28</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="F27" s="14" t="s">
         <v>25</v>
@@ -1816,102 +1838,102 @@
         <v>30</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="30">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="30.75">
       <c r="A28" s="14" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B28" s="15" t="s">
         <v>86</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D28" s="14" t="s">
         <v>23</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="F28" s="14" t="s">
         <v>25</v>
       </c>
       <c r="G28" s="13" t="s">
-        <v>89</v>
+        <v>49</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="30">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="30.75">
       <c r="A29" s="14" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B29" s="15" t="s">
         <v>86</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="D29" s="14" t="s">
         <v>17</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="F29" s="14" t="s">
         <v>19</v>
       </c>
       <c r="G29" s="13" t="s">
-        <v>89</v>
+        <v>20</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>89</v>
+        <v>110</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="27" customHeight="1">
       <c r="A30" s="14" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="B30" s="15" t="s">
         <v>86</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="D30" s="14" t="s">
         <v>23</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="F30" s="14" t="s">
         <v>25</v>
       </c>
       <c r="G30" s="13" t="s">
-        <v>89</v>
+        <v>20</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>89</v>
+        <v>113</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="27.75" customHeight="1">
       <c r="A31" s="14" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="B31" s="15" t="s">
         <v>86</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="D31" s="14" t="s">
         <v>28</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="F31" s="14" t="s">
         <v>25</v>
@@ -1920,501 +1942,501 @@
         <v>30</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" hidden="1">
       <c r="A32" s="14" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="D32" s="14" t="s">
         <v>28</v>
       </c>
       <c r="E32" s="14" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="F32" s="14" t="s">
         <v>25</v>
       </c>
       <c r="G32" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" ht="30">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="30" hidden="1">
       <c r="A33" s="14" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="D33" s="14" t="s">
         <v>28</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="F33" s="14" t="s">
         <v>25</v>
       </c>
       <c r="G33" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" ht="30">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="30" hidden="1">
       <c r="A34" s="14" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="D34" s="14" t="s">
         <v>23</v>
       </c>
       <c r="E34" s="14" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="F34" s="14" t="s">
         <v>25</v>
       </c>
       <c r="G34" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" ht="30">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="30" hidden="1">
       <c r="A35" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="B35" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="B35" s="15" t="s">
-        <v>110</v>
-      </c>
       <c r="C35" s="14" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="D35" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E35" s="14" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="F35" s="14" t="s">
         <v>25</v>
       </c>
       <c r="G35" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" ht="30">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="30" hidden="1">
       <c r="A36" s="14" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="D36" s="14" t="s">
         <v>17</v>
       </c>
       <c r="E36" s="14" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="F36" s="14" t="s">
         <v>19</v>
       </c>
       <c r="G36" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" ht="30">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="30" hidden="1">
       <c r="A37" s="14" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="D37" s="14" t="s">
         <v>28</v>
       </c>
       <c r="E37" s="14" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="F37" s="14" t="s">
         <v>25</v>
       </c>
       <c r="G37" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" hidden="1">
       <c r="A38" s="14" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="D38" s="14" t="s">
         <v>23</v>
       </c>
       <c r="E38" s="14" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="F38" s="14" t="s">
         <v>25</v>
       </c>
       <c r="G38" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H38" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" hidden="1">
       <c r="A39" s="14" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="D39" s="14" t="s">
         <v>17</v>
       </c>
       <c r="E39" s="14" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="F39" s="14" t="s">
         <v>19</v>
       </c>
       <c r="G39" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" hidden="1">
       <c r="A40" s="14" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="D40" s="14" t="s">
         <v>23</v>
       </c>
       <c r="E40" s="14" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="F40" s="14" t="s">
         <v>19</v>
       </c>
       <c r="G40" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H40" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" hidden="1">
       <c r="A41" s="14" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="D41" s="14" t="s">
         <v>28</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="F41" s="14" t="s">
         <v>19</v>
       </c>
       <c r="G41" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H41" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" hidden="1">
       <c r="A42" s="14" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B42" s="15" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="D42" s="14" t="s">
         <v>17</v>
       </c>
       <c r="E42" s="14" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F42" s="14" t="s">
         <v>19</v>
       </c>
       <c r="G42" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H42" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" hidden="1">
       <c r="A43" s="14" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="B43" s="15" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="D43" s="14" t="s">
         <v>23</v>
       </c>
       <c r="E43" s="14" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="F43" s="14" t="s">
         <v>19</v>
       </c>
       <c r="G43" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H43" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" hidden="1">
       <c r="A44" s="14" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="B44" s="15" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="D44" s="14" t="s">
         <v>28</v>
       </c>
       <c r="E44" s="14" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="F44" s="14" t="s">
         <v>19</v>
       </c>
       <c r="G44" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H44" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" ht="30">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="30" hidden="1">
       <c r="A45" s="14" t="s">
+        <v>148</v>
+      </c>
+      <c r="B45" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="B45" s="15" t="s">
-        <v>134</v>
-      </c>
       <c r="C45" s="14" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="D45" s="14" t="s">
         <v>17</v>
       </c>
       <c r="E45" s="14" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="F45" s="14" t="s">
         <v>19</v>
       </c>
       <c r="G45" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H45" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" ht="30">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="30" hidden="1">
       <c r="A46" s="14" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="B46" s="15" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="D46" s="14" t="s">
         <v>28</v>
       </c>
       <c r="E46" s="14" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="F46" s="14" t="s">
         <v>25</v>
       </c>
       <c r="G46" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H46" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" hidden="1">
       <c r="A47" s="14" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="B47" s="15" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="D47" s="14" t="s">
         <v>23</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="F47" s="14" t="s">
         <v>25</v>
       </c>
       <c r="G47" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H47" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" hidden="1">
       <c r="A48" s="14" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="B48" s="15" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="D48" s="14" t="s">
         <v>17</v>
       </c>
       <c r="E48" s="14" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="F48" s="14" t="s">
         <v>19</v>
       </c>
       <c r="G48" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H48" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" hidden="1">
       <c r="A49" s="14" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="B49" s="15" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="D49" s="14" t="s">
         <v>23</v>
       </c>
       <c r="E49" s="14" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="F49" s="14" t="s">
         <v>25</v>
       </c>
       <c r="G49" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H49" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" ht="30">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="30" hidden="1">
       <c r="A50" s="14" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="D50" s="14" t="s">
         <v>28</v>
       </c>
       <c r="E50" s="14" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="F50" s="14" t="s">
         <v>25</v>
       </c>
       <c r="G50" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H50" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -3279,6 +3301,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A4:H50" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Onda 3"/>
+      </filters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:H50">
       <sortCondition ref="B4:B50"/>
     </sortState>
@@ -3339,85 +3366,85 @@
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1">
       <c r="A1" s="20" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="B1" s="23"/>
     </row>
     <row r="2" spans="1:8" ht="39.950000000000003" customHeight="1">
       <c r="A2" s="7" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="39.950000000000003" customHeight="1">
       <c r="A3" s="9" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="39.950000000000003" customHeight="1">
       <c r="A4" s="7" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="39.950000000000003" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="39.950000000000003" customHeight="1">
       <c r="A6" s="7" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="39.950000000000003" customHeight="1">
       <c r="A7" s="9" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="39.950000000000003" customHeight="1">
       <c r="A8" s="7" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="39.950000000000003" customHeight="1">
       <c r="A9" s="9" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="39.950000000000003" customHeight="1">
       <c r="A10" s="7" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="22" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="B12" s="23"/>
       <c r="C12" s="23"/>
@@ -3430,7 +3457,7 @@
     <row r="13" spans="1:8">
       <c r="A13" s="3"/>
       <c r="B13" s="21" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="C13" s="23"/>
       <c r="D13" s="23"/>
@@ -3442,7 +3469,7 @@
     <row r="14" spans="1:8">
       <c r="A14" s="4"/>
       <c r="B14" s="21" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="C14" s="23"/>
       <c r="D14" s="23"/>
@@ -3454,7 +3481,7 @@
     <row r="15" spans="1:8">
       <c r="A15" s="5"/>
       <c r="B15" s="21" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="C15" s="23"/>
       <c r="D15" s="23"/>
@@ -3465,7 +3492,7 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="22" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="B17" s="23"/>
       <c r="C17" s="23"/>
@@ -3480,7 +3507,7 @@
         <v>9</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="C18" s="23"/>
       <c r="D18" s="23"/>
@@ -3494,7 +3521,7 @@
         <v>11</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="C19" s="23"/>
       <c r="D19" s="23"/>
@@ -3508,7 +3535,7 @@
         <v>13</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="C20" s="23"/>
       <c r="D20" s="23"/>
@@ -3535,6 +3562,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="d90de4e3-1570-4373-8742-4e5b70768c2c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100069CEBA7CDA2B54A9B4CB9D08A57C2BE" ma:contentTypeVersion="14" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="4076db77eab4abd82fb5a98d0e08ed94">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="d90de4e3-1570-4373-8742-4e5b70768c2c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c9ec4751c483cff2354015c975db5e37" ns3:_="">
     <xsd:import namespace="d90de4e3-1570-4373-8742-4e5b70768c2c"/>
@@ -3742,31 +3786,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="d90de4e3-1570-4373-8742-4e5b70768c2c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F54BD295-47E6-4D5E-AB8C-AB6A369202DB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8C9EAED-E792-4EBD-8FE5-A88413F06C36}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8C9EAED-E792-4EBD-8FE5-A88413F06C36}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0FA79B10-923E-46FD-992E-6B2FB513113C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0FA79B10-923E-46FD-992E-6B2FB513113C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F54BD295-47E6-4D5E-AB8C-AB6A369202DB}"/>
 </file>
</xml_diff>